<commit_message>
Added RDF data schemes, fixed xlsx-spreadsheets and visual schemes for food-table07-12
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/food-table08.xlsx
+++ b/sources/table_normalization/xlsx/food-table08.xlsx
@@ -228,7 +228,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -375,34 +375,34 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -891,24 +891,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="32.25" customHeight="1">
-      <c r="A1" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="13" t="s">
+      <c r="A1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14" t="s">
+      <c r="E1" s="17"/>
+      <c r="F1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="14"/>
-      <c r="H1" s="15" t="s">
+      <c r="G1" s="17"/>
+      <c r="H1" s="13" t="s">
         <v>5</v>
       </c>
     </row>
@@ -916,13 +916,13 @@
       <c r="A2" s="16"/>
       <c r="B2" s="16"/>
       <c r="C2" s="16"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17" t="s">
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="17"/>
-      <c r="H2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="14"/>
     </row>
     <row r="3" spans="1:8" ht="15.5">
       <c r="A3" s="16"/>
@@ -940,7 +940,7 @@
       <c r="G3" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="18"/>
+      <c r="H3" s="14"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="1" t="s">

</xml_diff>